<commit_message>
Support of more priorities, lambda value integrated, lots of bugfixes
</commit_message>
<xml_diff>
--- a/input/sample_coordinates.xlsx
+++ b/input/sample_coordinates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25427"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uibkacat-my.sharepoint.com/personal/benedikt_schenk_student_uibk_ac_at/Documents/Dokumente/UNI/bachelor/git/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{54762E30-87BC-4E04-AA38-374D7B6D3FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA5B71F8-65E6-4E28-9892-63D6E75B2DDF}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{54762E30-87BC-4E04-AA38-374D7B6D3FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A7BB1CC-6892-4278-8E6A-B769CA69A9F3}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="guides" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
   <si>
     <t>Guide</t>
   </si>
@@ -64,21 +64,9 @@
     <t>47.68250689894895, 11.576204060472987</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>47.2703660939085, 11.402158497018387</t>
   </si>
   <si>
-    <t>05234 Axams</t>
-  </si>
-  <si>
     <t>47.231910185690694, 11.280378993780598</t>
   </si>
   <si>
@@ -86,6 +74,30 @@
   </si>
   <si>
     <t>47.30592192560842, 11.067529601164987</t>
+  </si>
+  <si>
+    <t>Innsbruck</t>
+  </si>
+  <si>
+    <t>47.26837544415054, 11.39192245635583</t>
+  </si>
+  <si>
+    <t>Sebastian</t>
+  </si>
+  <si>
+    <t>Frederik</t>
+  </si>
+  <si>
+    <t>Jonas</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Daisy</t>
+  </si>
+  <si>
+    <t>5234 Axams</t>
   </si>
 </sst>
 </file>
@@ -929,13 +941,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="43.7265625" customWidth="1"/>
+    <col min="2" max="2" width="43.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -946,9 +958,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
@@ -957,26 +969,48 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -987,14 +1021,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.81640625" customWidth="1"/>
-    <col min="2" max="2" width="44.81640625" customWidth="1"/>
+    <col min="1" max="1" width="21.84375" customWidth="1"/>
+    <col min="2" max="2" width="44.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -1002,7 +1036,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1010,12 +1044,20 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>